<commit_message>
add screenshot on failure, ci/cd config, parallel execution
</commit_message>
<xml_diff>
--- a/data/DataUser.xlsx
+++ b/data/DataUser.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\injas\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CodeProject\Java\MyProject\CucumberBDDProject\CucumberMiniFramework\cucumber_hybrid_framework\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8C511810-91BB-4BD0-B865-D38C096784CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{552F43E7-AC4F-4B7F-8D2B-7F2024B285C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{31CA0C65-8FEB-46D4-AF69-AD6F97F4B75D}"/>
   </bookViews>
@@ -17,7 +17,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -36,30 +36,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>EMAIL</t>
   </si>
   <si>
     <t>PASSWORD</t>
-  </si>
-  <si>
-    <t>chieko.gibson@gmail.com</t>
-  </si>
-  <si>
-    <t>Of3%BGOK</t>
-  </si>
-  <si>
-    <t>sheena.jacobi@gmail.com</t>
-  </si>
-  <si>
-    <t>Hu7@7LD&amp;</t>
-  </si>
-  <si>
-    <t>creola.vandervort@gmail.com</t>
-  </si>
-  <si>
-    <t>Aq0%3MHB</t>
   </si>
   <si>
     <t>reid.cartwright@hotmail.com</t>
@@ -78,7 +60,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -444,55 +425,35 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{290CBC4D-1AFC-4B6D-8F9B-23F8520A0F28}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="0">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="s" s="0">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="s" s="0">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>5</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="B6" t="s" s="0">
-        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>